<commit_message>
Correction for lead + graphs improvements
</commit_message>
<xml_diff>
--- a/data/data_metals.xlsx
+++ b/data/data_metals.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca0-my.sharepoint.com/personal/marin_pellan_polymtlus_ca/Documents/Desktop/POST_DOC/Project/plca_metals_github/plca_metals/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1244" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6C4A5D2-D011-425E-8BF3-9A23DBBAA497}"/>
+  <xr:revisionPtr revIDLastSave="1247" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFA5159E-BAA4-4612-8331-3FB0E592F1FD}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -15425,22 +15425,22 @@
         <v>74</v>
       </c>
       <c r="G15">
-        <v>11444292.4227354</v>
+        <v>11431.7949327354</v>
       </c>
       <c r="H15">
-        <v>13897264.3387175</v>
+        <v>13882.0881342231</v>
       </c>
       <c r="I15">
-        <v>15673836.0626311</v>
+        <v>15656.719791723401</v>
       </c>
       <c r="J15">
-        <v>17503394.648657199</v>
+        <v>17484.2804481887</v>
       </c>
       <c r="K15">
-        <v>19553837.856053699</v>
+        <v>19532.484513790001</v>
       </c>
       <c r="L15">
-        <v>21726419.243699301</v>
+        <v>21702.693381304001</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Improvements for last modifications before submission
</commit_message>
<xml_diff>
--- a/data/data_metals.xlsx
+++ b/data/data_metals.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="1247" documentId="11_F25DC773A252ABDACC104887411C794C5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFA5159E-BAA4-4612-8331-3FB0E592F1FD}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>